<commit_message>
fix(encoding): set response.encoding to utf-8 and add curly quote test
</commit_message>
<xml_diff>
--- a/sample_output.xlsx
+++ b/sample_output.xlsx
@@ -522,7 +522,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SP-41187</t>
+          <t>SP-68896</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -556,14 +556,14 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>SP-48301</t>
+          <t>SP-64708</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -597,14 +597,14 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>SP-99651</t>
+          <t>SP-06375</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -638,14 +638,14 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>SP-94965</t>
+          <t>SP-12837</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -679,14 +679,14 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>SP-72113</t>
+          <t>SP-15702</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -720,14 +720,14 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>SP-54787</t>
+          <t>SP-68188</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -761,14 +761,14 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>SP-39394</t>
+          <t>SP-44550</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -802,14 +802,14 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>SP-37513</t>
+          <t>SP-64925</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -843,14 +843,14 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>SP-84062</t>
+          <t>SP-95686</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -884,14 +884,14 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SP-66559</t>
+          <t>SP-83014</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -925,14 +925,14 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SP-89728</t>
+          <t>SP-20710</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -966,14 +966,14 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>SP-06668</t>
+          <t>SP-33561</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1007,14 +1007,14 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>SP-55931</t>
+          <t>SP-88209</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1048,14 +1048,14 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>SP-47479</t>
+          <t>SP-39335</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1089,14 +1089,14 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>SP-80672</t>
+          <t>SP-64336</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1130,14 +1130,14 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>SP-97562</t>
+          <t>SP-29437</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1171,14 +1171,14 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>SP-70233</t>
+          <t>SP-07821</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1212,14 +1212,14 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>SP-87389</t>
+          <t>SP-35935</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1253,14 +1253,14 @@
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>SP-61276</t>
+          <t>SP-10909</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1294,14 +1294,14 @@
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>SP-37375</t>
+          <t>SP-41357</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1335,14 +1335,14 @@
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:48</t>
+          <t>2026-10-03 14:50:09</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>SP-69565</t>
+          <t>SP-38575</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1376,14 +1376,14 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>SP-65205</t>
+          <t>SP-43076</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1417,14 +1417,14 @@
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>SP-87315</t>
+          <t>SP-58368</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1458,14 +1458,14 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>SP-45825</t>
+          <t>SP-90951</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1499,14 +1499,14 @@
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>SP-90554</t>
+          <t>SP-50129</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1540,14 +1540,14 @@
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>SP-14137</t>
+          <t>SP-23151</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1581,14 +1581,14 @@
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>SP-86097</t>
+          <t>SP-46061</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1622,14 +1622,14 @@
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>SP-04890</t>
+          <t>SP-33302</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1663,19 +1663,19 @@
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>SP-25284</t>
+          <t>SP-58620</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Worlds Elsewhere: Journeys Around Shakespeareâs Globe</t>
+          <t>Worlds Elsewhere: Journeys Around Shakespeare’s Globe</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
@@ -1704,14 +1704,14 @@
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>SP-59068</t>
+          <t>SP-44045</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1745,14 +1745,14 @@
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>SP-11142</t>
+          <t>SP-42670</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1786,14 +1786,14 @@
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>SP-31902</t>
+          <t>SP-58159</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1827,14 +1827,14 @@
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>SP-53620</t>
+          <t>SP-98235</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1868,14 +1868,14 @@
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>SP-44997</t>
+          <t>SP-18284</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1909,14 +1909,14 @@
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>SP-81333</t>
+          <t>SP-82144</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1950,14 +1950,14 @@
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>SP-59858</t>
+          <t>SP-83357</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1991,14 +1991,14 @@
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>SP-03103</t>
+          <t>SP-35743</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -2032,14 +2032,14 @@
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>SP-64403</t>
+          <t>SP-74073</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -2073,14 +2073,14 @@
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>SP-06320</t>
+          <t>SP-00046</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -2114,14 +2114,14 @@
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>SP-90649</t>
+          <t>SP-10194</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:54:49</t>
+          <t>2026-10-03 14:50:11</t>
         </is>
       </c>
     </row>

</xml_diff>